<commit_message>
Add visual dashboards v2 and on-demand spreadsheet generator
Upgrade the 7 workbooks with branded dashboards, charts and KPI
cards, and ship a client-side generator to customize and download.
</commit_message>
<xml_diff>
--- a/public/planilhas/01_controle_financeiro_pessoal.xlsx
+++ b/public/planilhas/01_controle_financeiro_pessoal.xlsx
@@ -18,13 +18,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="166" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="167" formatCode="MMM/YYYY"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,12 +36,18 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000A1322"/>
-      <sz val="18"/>
+      <color rgb="00C99C66"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="005C6B82"/>
+      <b val="1"/>
+      <color rgb="000A1322"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="008593A8"/>
       <sz val="11"/>
     </font>
     <font>
@@ -51,22 +58,52 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="000A1322"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008593A8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008593A8"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000A1322"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="18"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="000A1322"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
-      <sz val="13"/>
+      <color rgb="00C99C66"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="11"/>
     </font>
     <font>
       <i val="1"/>
-      <color rgb="005C6B82"/>
+      <color rgb="008593A8"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -80,7 +117,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6F1EA"/>
+        <fgColor rgb="00F8F4EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8D0A8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECFDF5"/>
       </patternFill>
     </fill>
   </fills>
@@ -94,37 +156,56 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D0D7DE"/>
+        <color rgb="00E5E7EB"/>
       </left>
       <right style="thin">
-        <color rgb="00D0D7DE"/>
+        <color rgb="00E5E7EB"/>
       </right>
       <top style="thin">
-        <color rgb="00D0D7DE"/>
+        <color rgb="00E5E7EB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D0D7DE"/>
+        <color rgb="00E5E7EB"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -266,9 +347,9 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>3</col>
+      <col>5</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>9</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="3600000"/>
@@ -578,220 +659,361 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Trust Excel · Painel Financeiro</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>TRUST EXCEL  ·  TRUST CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Totais automáticos do mês atual + gastos por categoria</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+          <t>Dashboard Financeiro Pessoal</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Totais do mês · ranking de categorias · gráfico visual</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Mês de referência</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B5" s="5" t="n">
         <v>46204</v>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Total Entradas</t>
-        </is>
-      </c>
-      <c r="B6" s="5">
-        <f>SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!D:D,"Entrada",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0))</f>
-        <v/>
-      </c>
-    </row>
+    <row r="6"/>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Total Saídas</t>
-        </is>
-      </c>
-      <c r="B7" s="5">
-        <f>SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Saldo do mês</t>
-        </is>
-      </c>
-      <c r="B8" s="6">
-        <f>B6-B7</f>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL ENTRADAS</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL SAÍDAS</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>SALDO DO MÊS</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>TAXA DE GASTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="7">
+        <f>SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!D:D,"Entrada",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0))</f>
+        <v/>
+      </c>
+      <c r="C8" s="7">
+        <f>SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0))</f>
+        <v/>
+      </c>
+      <c r="E8" s="8">
+        <f>A8-C8</f>
+        <v/>
+      </c>
+      <c r="G8" s="9">
+        <f>IFERROR(C8/A8,0)</f>
         <v/>
       </c>
     </row>
     <row r="9"/>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Gastos por categoria</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>GASTOS POR CATEGORIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Total Saídas</t>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>% do gasto</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Barra</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9">
-        <f>IF(CATEGORIAS!A5="","",CATEGORIAS!A5)</f>
-        <v/>
-      </c>
-      <c r="B12" s="5">
-        <f>IF(A12="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A12,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0)))</f>
+      <c r="A12" s="12">
+        <f>IF(CATEGORIAS!A6="","",CATEGORIAS!A6)</f>
+        <v/>
+      </c>
+      <c r="B12" s="13">
+        <f>IF(A12="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A12,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0)))</f>
+        <v/>
+      </c>
+      <c r="C12" s="14">
+        <f>IF(OR(A12="",$C$8=0),"",B12/$C$8)</f>
+        <v/>
+      </c>
+      <c r="D12" s="12">
+        <f>IF(C12="","",REPT("█",ROUNDDOWN(C12*20,0))&amp;REPT("░",20-ROUNDDOWN(C12*20,0)))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9">
-        <f>IF(CATEGORIAS!A6="","",CATEGORIAS!A6)</f>
-        <v/>
-      </c>
-      <c r="B13" s="5">
-        <f>IF(A13="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A13,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0)))</f>
+      <c r="A13" s="15">
+        <f>IF(CATEGORIAS!A7="","",CATEGORIAS!A7)</f>
+        <v/>
+      </c>
+      <c r="B13" s="16">
+        <f>IF(A13="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A13,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0)))</f>
+        <v/>
+      </c>
+      <c r="C13" s="17">
+        <f>IF(OR(A13="",$C$8=0),"",B13/$C$8)</f>
+        <v/>
+      </c>
+      <c r="D13" s="15">
+        <f>IF(C13="","",REPT("█",ROUNDDOWN(C13*20,0))&amp;REPT("░",20-ROUNDDOWN(C13*20,0)))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9">
-        <f>IF(CATEGORIAS!A7="","",CATEGORIAS!A7)</f>
-        <v/>
-      </c>
-      <c r="B14" s="5">
-        <f>IF(A14="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A14,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0)))</f>
+      <c r="A14" s="12">
+        <f>IF(CATEGORIAS!A8="","",CATEGORIAS!A8)</f>
+        <v/>
+      </c>
+      <c r="B14" s="13">
+        <f>IF(A14="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A14,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0)))</f>
+        <v/>
+      </c>
+      <c r="C14" s="14">
+        <f>IF(OR(A14="",$C$8=0),"",B14/$C$8)</f>
+        <v/>
+      </c>
+      <c r="D14" s="12">
+        <f>IF(C14="","",REPT("█",ROUNDDOWN(C14*20,0))&amp;REPT("░",20-ROUNDDOWN(C14*20,0)))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9">
-        <f>IF(CATEGORIAS!A8="","",CATEGORIAS!A8)</f>
-        <v/>
-      </c>
-      <c r="B15" s="5">
-        <f>IF(A15="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A15,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0)))</f>
+      <c r="A15" s="15">
+        <f>IF(CATEGORIAS!A9="","",CATEGORIAS!A9)</f>
+        <v/>
+      </c>
+      <c r="B15" s="16">
+        <f>IF(A15="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A15,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0)))</f>
+        <v/>
+      </c>
+      <c r="C15" s="17">
+        <f>IF(OR(A15="",$C$8=0),"",B15/$C$8)</f>
+        <v/>
+      </c>
+      <c r="D15" s="15">
+        <f>IF(C15="","",REPT("█",ROUNDDOWN(C15*20,0))&amp;REPT("░",20-ROUNDDOWN(C15*20,0)))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9">
-        <f>IF(CATEGORIAS!A9="","",CATEGORIAS!A9)</f>
-        <v/>
-      </c>
-      <c r="B16" s="5">
-        <f>IF(A16="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A16,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0)))</f>
+      <c r="A16" s="12">
+        <f>IF(CATEGORIAS!A10="","",CATEGORIAS!A10)</f>
+        <v/>
+      </c>
+      <c r="B16" s="13">
+        <f>IF(A16="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A16,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0)))</f>
+        <v/>
+      </c>
+      <c r="C16" s="14">
+        <f>IF(OR(A16="",$C$8=0),"",B16/$C$8)</f>
+        <v/>
+      </c>
+      <c r="D16" s="12">
+        <f>IF(C16="","",REPT("█",ROUNDDOWN(C16*20,0))&amp;REPT("░",20-ROUNDDOWN(C16*20,0)))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9">
-        <f>IF(CATEGORIAS!A10="","",CATEGORIAS!A10)</f>
-        <v/>
-      </c>
-      <c r="B17" s="5">
-        <f>IF(A17="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A17,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0)))</f>
+      <c r="A17" s="15">
+        <f>IF(CATEGORIAS!A11="","",CATEGORIAS!A11)</f>
+        <v/>
+      </c>
+      <c r="B17" s="16">
+        <f>IF(A17="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A17,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0)))</f>
+        <v/>
+      </c>
+      <c r="C17" s="17">
+        <f>IF(OR(A17="",$C$8=0),"",B17/$C$8)</f>
+        <v/>
+      </c>
+      <c r="D17" s="15">
+        <f>IF(C17="","",REPT("█",ROUNDDOWN(C17*20,0))&amp;REPT("░",20-ROUNDDOWN(C17*20,0)))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9">
-        <f>IF(CATEGORIAS!A11="","",CATEGORIAS!A11)</f>
-        <v/>
-      </c>
-      <c r="B18" s="5">
-        <f>IF(A18="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A18,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0)))</f>
+      <c r="A18" s="12">
+        <f>IF(CATEGORIAS!A12="","",CATEGORIAS!A12)</f>
+        <v/>
+      </c>
+      <c r="B18" s="13">
+        <f>IF(A18="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A18,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0)))</f>
+        <v/>
+      </c>
+      <c r="C18" s="14">
+        <f>IF(OR(A18="",$C$8=0),"",B18/$C$8)</f>
+        <v/>
+      </c>
+      <c r="D18" s="12">
+        <f>IF(C18="","",REPT("█",ROUNDDOWN(C18*20,0))&amp;REPT("░",20-ROUNDDOWN(C18*20,0)))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="9">
-        <f>IF(CATEGORIAS!A12="","",CATEGORIAS!A12)</f>
-        <v/>
-      </c>
-      <c r="B19" s="5">
-        <f>IF(A19="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A19,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0)))</f>
+      <c r="A19" s="15">
+        <f>IF(CATEGORIAS!A13="","",CATEGORIAS!A13)</f>
+        <v/>
+      </c>
+      <c r="B19" s="16">
+        <f>IF(A19="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A19,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0)))</f>
+        <v/>
+      </c>
+      <c r="C19" s="17">
+        <f>IF(OR(A19="",$C$8=0),"",B19/$C$8)</f>
+        <v/>
+      </c>
+      <c r="D19" s="15">
+        <f>IF(C19="","",REPT("█",ROUNDDOWN(C19*20,0))&amp;REPT("░",20-ROUNDDOWN(C19*20,0)))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9">
-        <f>IF(CATEGORIAS!A13="","",CATEGORIAS!A13)</f>
-        <v/>
-      </c>
-      <c r="B20" s="5">
-        <f>IF(A20="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A20,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0)))</f>
+      <c r="A20" s="12">
+        <f>IF(CATEGORIAS!A14="","",CATEGORIAS!A14)</f>
+        <v/>
+      </c>
+      <c r="B20" s="13">
+        <f>IF(A20="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A20,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0)))</f>
+        <v/>
+      </c>
+      <c r="C20" s="14">
+        <f>IF(OR(A20="",$C$8=0),"",B20/$C$8)</f>
+        <v/>
+      </c>
+      <c r="D20" s="12">
+        <f>IF(C20="","",REPT("█",ROUNDDOWN(C20*20,0))&amp;REPT("░",20-ROUNDDOWN(C20*20,0)))</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9">
-        <f>IF(CATEGORIAS!A14="","",CATEGORIAS!A14)</f>
-        <v/>
-      </c>
-      <c r="B21" s="5">
-        <f>IF(A21="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A21,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0)))</f>
+      <c r="A21" s="15">
+        <f>IF(CATEGORIAS!A15="","",CATEGORIAS!A15)</f>
+        <v/>
+      </c>
+      <c r="B21" s="16">
+        <f>IF(A21="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A21,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0)))</f>
+        <v/>
+      </c>
+      <c r="C21" s="17">
+        <f>IF(OR(A21="",$C$8=0),"",B21/$C$8)</f>
+        <v/>
+      </c>
+      <c r="D21" s="15">
+        <f>IF(C21="","",REPT("█",ROUNDDOWN(C21*20,0))&amp;REPT("░",20-ROUNDDOWN(C21*20,0)))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9">
-        <f>IF(CATEGORIAS!A15="","",CATEGORIAS!A15)</f>
-        <v/>
-      </c>
-      <c r="B22" s="5">
-        <f>IF(A22="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A22,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$4,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$4,0)))</f>
+      <c r="A22" s="12">
+        <f>IF(CATEGORIAS!A16="","",CATEGORIAS!A16)</f>
+        <v/>
+      </c>
+      <c r="B22" s="13">
+        <f>IF(A22="","",SUMIFS(LANCAMENTOS!E:E,LANCAMENTOS!B:B,A22,LANCAMENTOS!D:D,"Saída",LANCAMENTOS!A:A,"&gt;="&amp;$B$5,LANCAMENTOS!A:A,"&lt;="&amp;EOMONTH($B$5,0)))</f>
+        <v/>
+      </c>
+      <c r="C22" s="14">
+        <f>IF(OR(A22="",$C$8=0),"",B22/$C$8)</f>
+        <v/>
+      </c>
+      <c r="D22" s="12">
+        <f>IF(C22="","",REPT("█",ROUNDDOWN(C22*20,0))&amp;REPT("░",20-ROUNDDOWN(C22*20,0)))</f>
         <v/>
       </c>
     </row>
     <row r="23"/>
     <row r="24"/>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Automação TrustCorp: preencha LANCAMENTOS; o PAINEL recalcula sozinho. Use lista suspensa em Categoria e Tipo.</t>
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>INSIGHT AUTOMÁTICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="19">
+        <f>CONCATENATE("Maior categoria de gasto: ",INDEX(A12:A22,MATCH(MAX(B12:B22),B12:B22,0))," com ",TEXT(MAX(B12:B22),"R$ #,##0.00")," (",TEXT(MAX(C12:C22),"0%")," do total).")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>Automação TrustCorp: preencha LANCAMENTOS com listas suspensas. O dashboard recalcula totais, ranking, barras e gráfico.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+  <mergeCells count="4">
+    <mergeCell ref="A26:E27"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <conditionalFormatting sqref="B12:B22">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00FEF3C7"/>
+        <color rgb="00EF4444"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -803,114 +1025,122 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Trust Excel · Categorias</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>TRUST EXCEL  ·  TRUST CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Lista-mestre para validação de lançamentos</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+          <t>Categorias</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Lista-mestre para validação dos lançamentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Moradia</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Alimentação</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Transporte</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Lazer</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Assinaturas</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Saúde</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Educação</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Salário</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Freelance</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Investimentos</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Outros</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A3:B3"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
@@ -924,578 +1154,786 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Trust Excel · Controle Financeiro Pessoal</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>TRUST EXCEL  ·  TRUST CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Lançamentos do mês · tabelas e listas suspensas</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+          <t>Lançamentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Preencha aqui · o painel atualiza sozinho</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="11" t="n">
+    <row r="6">
+      <c r="A6" s="22" t="n">
         <v>46205</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Salário</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Salário mensal</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D6" s="23" t="inlineStr">
         <is>
           <t>Entrada</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n">
-        <v>8500</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="n">
+      <c r="E6" s="16" t="n">
+        <v>9200</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="n">
         <v>46206</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Moradia</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Aluguel</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Aluguel + condomínio</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E6" s="5" t="n">
-        <v>2200</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="E7" s="16" t="n">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="n">
         <v>46207</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Alimentação</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Mercado</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Mercado mensal</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n">
-        <v>640.5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="n">
+      <c r="E8" s="16" t="n">
+        <v>780.4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="n">
         <v>46208</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Assinaturas</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Streaming + software</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Softwares e streaming</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n">
-        <v>189.9</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="E9" s="16" t="n">
+        <v>219.9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="n">
         <v>46209</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Transporte</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Combustível</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Combustível / app</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E9" s="5" t="n">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="n">
+      <c r="E10" s="16" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="n">
         <v>46210</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Freelance</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>Projeto cliente A</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D11" s="23" t="inlineStr">
         <is>
           <t>Entrada</t>
         </is>
       </c>
-      <c r="E10" s="5" t="n">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="E11" s="16" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="n">
         <v>46211</v>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Lazer</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>Restaurante</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D12" s="24" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E11" s="5" t="n">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="n">
+      <c r="E12" s="16" t="n">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="n">
         <v>46212</v>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>Saúde</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Farmácia</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>Farmácia / consulta</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E12" s="5" t="n">
-        <v>95.40000000000001</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="n">
+      <c r="E13" s="16" t="n">
+        <v>145.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="n">
         <v>46214</v>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Alimentação</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>Delivery</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D14" s="24" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E13" s="5" t="n">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="11" t="n">
+      <c r="E14" s="16" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="n">
         <v>46216</v>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>Investimentos</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>Aporte mensal</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D15" s="24" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E14" s="5" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="5" t="n"/>
+      <c r="E15" s="16" t="n">
+        <v>800</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="9" t="n"/>
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9" t="n"/>
-      <c r="E16" s="5" t="n"/>
+      <c r="A16" s="22" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Educação</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Curso / livro</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="n">
+        <v>189</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="5" t="n"/>
+      <c r="A17" s="22" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>Bônus entrega</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="n">
+        <v>650</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="5" t="n"/>
+      <c r="A18" s="22" t="n"/>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="16" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="5" t="n"/>
+      <c r="A19" s="22" t="n"/>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="16" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n"/>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="5" t="n"/>
+      <c r="A20" s="22" t="n"/>
+      <c r="B20" s="15" t="n"/>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="16" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n"/>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="5" t="n"/>
+      <c r="A21" s="22" t="n"/>
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="16" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n"/>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="5" t="n"/>
+      <c r="A22" s="22" t="n"/>
+      <c r="B22" s="15" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="16" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="5" t="n"/>
+      <c r="A23" s="22" t="n"/>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="16" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="n"/>
-      <c r="B24" s="9" t="n"/>
-      <c r="C24" s="9" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="5" t="n"/>
+      <c r="A24" s="22" t="n"/>
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="16" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n"/>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="9" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="5" t="n"/>
+      <c r="A25" s="22" t="n"/>
+      <c r="B25" s="15" t="n"/>
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="15" t="n"/>
+      <c r="E25" s="16" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="n"/>
-      <c r="B26" s="9" t="n"/>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="5" t="n"/>
+      <c r="A26" s="22" t="n"/>
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="16" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n"/>
-      <c r="B27" s="9" t="n"/>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="5" t="n"/>
+      <c r="A27" s="22" t="n"/>
+      <c r="B27" s="15" t="n"/>
+      <c r="C27" s="15" t="n"/>
+      <c r="D27" s="15" t="n"/>
+      <c r="E27" s="16" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="n"/>
-      <c r="B28" s="9" t="n"/>
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="5" t="n"/>
+      <c r="A28" s="22" t="n"/>
+      <c r="B28" s="15" t="n"/>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="16" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n"/>
-      <c r="B29" s="9" t="n"/>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="5" t="n"/>
+      <c r="A29" s="22" t="n"/>
+      <c r="B29" s="15" t="n"/>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="16" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="n"/>
-      <c r="B30" s="9" t="n"/>
-      <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="5" t="n"/>
+      <c r="A30" s="22" t="n"/>
+      <c r="B30" s="15" t="n"/>
+      <c r="C30" s="15" t="n"/>
+      <c r="D30" s="15" t="n"/>
+      <c r="E30" s="16" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n"/>
-      <c r="B31" s="9" t="n"/>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="9" t="n"/>
-      <c r="E31" s="5" t="n"/>
+      <c r="A31" s="22" t="n"/>
+      <c r="B31" s="15" t="n"/>
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="16" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="n"/>
-      <c r="B32" s="9" t="n"/>
-      <c r="C32" s="9" t="n"/>
-      <c r="D32" s="9" t="n"/>
-      <c r="E32" s="5" t="n"/>
+      <c r="A32" s="22" t="n"/>
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="16" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="n"/>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="9" t="n"/>
-      <c r="E33" s="5" t="n"/>
+      <c r="A33" s="22" t="n"/>
+      <c r="B33" s="15" t="n"/>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="15" t="n"/>
+      <c r="E33" s="16" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="n"/>
-      <c r="B34" s="9" t="n"/>
-      <c r="C34" s="9" t="n"/>
-      <c r="D34" s="9" t="n"/>
-      <c r="E34" s="5" t="n"/>
+      <c r="A34" s="22" t="n"/>
+      <c r="B34" s="15" t="n"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="16" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="n"/>
-      <c r="B35" s="9" t="n"/>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="9" t="n"/>
-      <c r="E35" s="5" t="n"/>
+      <c r="A35" s="22" t="n"/>
+      <c r="B35" s="15" t="n"/>
+      <c r="C35" s="15" t="n"/>
+      <c r="D35" s="15" t="n"/>
+      <c r="E35" s="16" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="n"/>
-      <c r="B36" s="9" t="n"/>
-      <c r="C36" s="9" t="n"/>
-      <c r="D36" s="9" t="n"/>
-      <c r="E36" s="5" t="n"/>
+      <c r="A36" s="22" t="n"/>
+      <c r="B36" s="15" t="n"/>
+      <c r="C36" s="15" t="n"/>
+      <c r="D36" s="15" t="n"/>
+      <c r="E36" s="16" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="n"/>
-      <c r="B37" s="9" t="n"/>
-      <c r="C37" s="9" t="n"/>
-      <c r="D37" s="9" t="n"/>
-      <c r="E37" s="5" t="n"/>
+      <c r="A37" s="22" t="n"/>
+      <c r="B37" s="15" t="n"/>
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="16" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="n"/>
-      <c r="B38" s="9" t="n"/>
-      <c r="C38" s="9" t="n"/>
-      <c r="D38" s="9" t="n"/>
-      <c r="E38" s="5" t="n"/>
+      <c r="A38" s="22" t="n"/>
+      <c r="B38" s="15" t="n"/>
+      <c r="C38" s="15" t="n"/>
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="16" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="n"/>
-      <c r="B39" s="9" t="n"/>
-      <c r="C39" s="9" t="n"/>
-      <c r="D39" s="9" t="n"/>
-      <c r="E39" s="5" t="n"/>
+      <c r="A39" s="22" t="n"/>
+      <c r="B39" s="15" t="n"/>
+      <c r="C39" s="15" t="n"/>
+      <c r="D39" s="15" t="n"/>
+      <c r="E39" s="16" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="n"/>
-      <c r="B40" s="9" t="n"/>
-      <c r="C40" s="9" t="n"/>
-      <c r="D40" s="9" t="n"/>
-      <c r="E40" s="5" t="n"/>
+      <c r="A40" s="22" t="n"/>
+      <c r="B40" s="15" t="n"/>
+      <c r="C40" s="15" t="n"/>
+      <c r="D40" s="15" t="n"/>
+      <c r="E40" s="16" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="n"/>
-      <c r="B41" s="9" t="n"/>
-      <c r="C41" s="9" t="n"/>
-      <c r="D41" s="9" t="n"/>
-      <c r="E41" s="5" t="n"/>
+      <c r="A41" s="22" t="n"/>
+      <c r="B41" s="15" t="n"/>
+      <c r="C41" s="15" t="n"/>
+      <c r="D41" s="15" t="n"/>
+      <c r="E41" s="16" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="n"/>
-      <c r="B42" s="9" t="n"/>
-      <c r="C42" s="9" t="n"/>
-      <c r="D42" s="9" t="n"/>
-      <c r="E42" s="5" t="n"/>
+      <c r="A42" s="22" t="n"/>
+      <c r="B42" s="15" t="n"/>
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="16" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="n"/>
-      <c r="B43" s="9" t="n"/>
-      <c r="C43" s="9" t="n"/>
-      <c r="D43" s="9" t="n"/>
-      <c r="E43" s="5" t="n"/>
+      <c r="A43" s="22" t="n"/>
+      <c r="B43" s="15" t="n"/>
+      <c r="C43" s="15" t="n"/>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="16" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="11" t="n"/>
-      <c r="B44" s="9" t="n"/>
-      <c r="C44" s="9" t="n"/>
-      <c r="D44" s="9" t="n"/>
-      <c r="E44" s="5" t="n"/>
+      <c r="A44" s="22" t="n"/>
+      <c r="B44" s="15" t="n"/>
+      <c r="C44" s="15" t="n"/>
+      <c r="D44" s="15" t="n"/>
+      <c r="E44" s="16" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="n"/>
-      <c r="B45" s="9" t="n"/>
-      <c r="C45" s="9" t="n"/>
-      <c r="D45" s="9" t="n"/>
-      <c r="E45" s="5" t="n"/>
+      <c r="A45" s="22" t="n"/>
+      <c r="B45" s="15" t="n"/>
+      <c r="C45" s="15" t="n"/>
+      <c r="D45" s="15" t="n"/>
+      <c r="E45" s="16" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="11" t="n"/>
-      <c r="B46" s="9" t="n"/>
-      <c r="C46" s="9" t="n"/>
-      <c r="D46" s="9" t="n"/>
-      <c r="E46" s="5" t="n"/>
+      <c r="A46" s="22" t="n"/>
+      <c r="B46" s="15" t="n"/>
+      <c r="C46" s="15" t="n"/>
+      <c r="D46" s="15" t="n"/>
+      <c r="E46" s="16" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="11" t="n"/>
-      <c r="B47" s="9" t="n"/>
-      <c r="C47" s="9" t="n"/>
-      <c r="D47" s="9" t="n"/>
-      <c r="E47" s="5" t="n"/>
+      <c r="A47" s="22" t="n"/>
+      <c r="B47" s="15" t="n"/>
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="16" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="n"/>
-      <c r="B48" s="9" t="n"/>
-      <c r="C48" s="9" t="n"/>
-      <c r="D48" s="9" t="n"/>
-      <c r="E48" s="5" t="n"/>
+      <c r="A48" s="22" t="n"/>
+      <c r="B48" s="15" t="n"/>
+      <c r="C48" s="15" t="n"/>
+      <c r="D48" s="15" t="n"/>
+      <c r="E48" s="16" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="n"/>
-      <c r="B49" s="9" t="n"/>
-      <c r="C49" s="9" t="n"/>
-      <c r="D49" s="9" t="n"/>
-      <c r="E49" s="5" t="n"/>
+      <c r="A49" s="22" t="n"/>
+      <c r="B49" s="15" t="n"/>
+      <c r="C49" s="15" t="n"/>
+      <c r="D49" s="15" t="n"/>
+      <c r="E49" s="16" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="n"/>
-      <c r="B50" s="9" t="n"/>
-      <c r="C50" s="9" t="n"/>
-      <c r="D50" s="9" t="n"/>
-      <c r="E50" s="5" t="n"/>
+      <c r="A50" s="22" t="n"/>
+      <c r="B50" s="15" t="n"/>
+      <c r="C50" s="15" t="n"/>
+      <c r="D50" s="15" t="n"/>
+      <c r="E50" s="16" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="n"/>
-      <c r="B51" s="9" t="n"/>
-      <c r="C51" s="9" t="n"/>
-      <c r="D51" s="9" t="n"/>
-      <c r="E51" s="5" t="n"/>
+      <c r="A51" s="22" t="n"/>
+      <c r="B51" s="15" t="n"/>
+      <c r="C51" s="15" t="n"/>
+      <c r="D51" s="15" t="n"/>
+      <c r="E51" s="16" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="11" t="n"/>
-      <c r="B52" s="9" t="n"/>
-      <c r="C52" s="9" t="n"/>
-      <c r="D52" s="9" t="n"/>
-      <c r="E52" s="5" t="n"/>
+      <c r="A52" s="22" t="n"/>
+      <c r="B52" s="15" t="n"/>
+      <c r="C52" s="15" t="n"/>
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="16" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="11" t="n"/>
-      <c r="B53" s="9" t="n"/>
-      <c r="C53" s="9" t="n"/>
-      <c r="D53" s="9" t="n"/>
-      <c r="E53" s="5" t="n"/>
+      <c r="A53" s="22" t="n"/>
+      <c r="B53" s="15" t="n"/>
+      <c r="C53" s="15" t="n"/>
+      <c r="D53" s="15" t="n"/>
+      <c r="E53" s="16" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="11" t="n"/>
-      <c r="B54" s="9" t="n"/>
-      <c r="C54" s="9" t="n"/>
-      <c r="D54" s="9" t="n"/>
-      <c r="E54" s="5" t="n"/>
+      <c r="A54" s="22" t="n"/>
+      <c r="B54" s="15" t="n"/>
+      <c r="C54" s="15" t="n"/>
+      <c r="D54" s="15" t="n"/>
+      <c r="E54" s="16" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="22" t="n"/>
+      <c r="B55" s="15" t="n"/>
+      <c r="C55" s="15" t="n"/>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="16" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="22" t="n"/>
+      <c r="B56" s="15" t="n"/>
+      <c r="C56" s="15" t="n"/>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="16" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="22" t="n"/>
+      <c r="B57" s="15" t="n"/>
+      <c r="C57" s="15" t="n"/>
+      <c r="D57" s="15" t="n"/>
+      <c r="E57" s="16" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="22" t="n"/>
+      <c r="B58" s="15" t="n"/>
+      <c r="C58" s="15" t="n"/>
+      <c r="D58" s="15" t="n"/>
+      <c r="E58" s="16" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="22" t="n"/>
+      <c r="B59" s="15" t="n"/>
+      <c r="C59" s="15" t="n"/>
+      <c r="D59" s="15" t="n"/>
+      <c r="E59" s="16" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="22" t="n"/>
+      <c r="B60" s="15" t="n"/>
+      <c r="C60" s="15" t="n"/>
+      <c r="D60" s="15" t="n"/>
+      <c r="E60" s="16" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="22" t="n"/>
+      <c r="B61" s="15" t="n"/>
+      <c r="C61" s="15" t="n"/>
+      <c r="D61" s="15" t="n"/>
+      <c r="E61" s="16" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="22" t="n"/>
+      <c r="B62" s="15" t="n"/>
+      <c r="C62" s="15" t="n"/>
+      <c r="D62" s="15" t="n"/>
+      <c r="E62" s="16" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="22" t="n"/>
+      <c r="B63" s="15" t="n"/>
+      <c r="C63" s="15" t="n"/>
+      <c r="D63" s="15" t="n"/>
+      <c r="E63" s="16" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="22" t="n"/>
+      <c r="B64" s="15" t="n"/>
+      <c r="C64" s="15" t="n"/>
+      <c r="D64" s="15" t="n"/>
+      <c r="E64" s="16" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="22" t="n"/>
+      <c r="B65" s="15" t="n"/>
+      <c r="C65" s="15" t="n"/>
+      <c r="D65" s="15" t="n"/>
+      <c r="E65" s="16" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="22" t="n"/>
+      <c r="B66" s="15" t="n"/>
+      <c r="C66" s="15" t="n"/>
+      <c r="D66" s="15" t="n"/>
+      <c r="E66" s="16" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="22" t="n"/>
+      <c r="B67" s="15" t="n"/>
+      <c r="C67" s="15" t="n"/>
+      <c r="D67" s="15" t="n"/>
+      <c r="E67" s="16" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="22" t="n"/>
+      <c r="B68" s="15" t="n"/>
+      <c r="C68" s="15" t="n"/>
+      <c r="D68" s="15" t="n"/>
+      <c r="E68" s="16" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="22" t="n"/>
+      <c r="B69" s="15" t="n"/>
+      <c r="C69" s="15" t="n"/>
+      <c r="D69" s="15" t="n"/>
+      <c r="E69" s="16" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="22" t="n"/>
+      <c r="B70" s="15" t="n"/>
+      <c r="C70" s="15" t="n"/>
+      <c r="D70" s="15" t="n"/>
+      <c r="E70" s="16" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="22" t="n"/>
+      <c r="B71" s="15" t="n"/>
+      <c r="C71" s="15" t="n"/>
+      <c r="D71" s="15" t="n"/>
+      <c r="E71" s="16" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="22" t="n"/>
+      <c r="B72" s="15" t="n"/>
+      <c r="C72" s="15" t="n"/>
+      <c r="D72" s="15" t="n"/>
+      <c r="E72" s="16" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="22" t="n"/>
+      <c r="B73" s="15" t="n"/>
+      <c r="C73" s="15" t="n"/>
+      <c r="D73" s="15" t="n"/>
+      <c r="E73" s="16" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="22" t="n"/>
+      <c r="B74" s="15" t="n"/>
+      <c r="C74" s="15" t="n"/>
+      <c r="D74" s="15" t="n"/>
+      <c r="E74" s="16" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="22" t="n"/>
+      <c r="B75" s="15" t="n"/>
+      <c r="C75" s="15" t="n"/>
+      <c r="D75" s="15" t="n"/>
+      <c r="E75" s="16" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="22" t="n"/>
+      <c r="B76" s="15" t="n"/>
+      <c r="C76" s="15" t="n"/>
+      <c r="D76" s="15" t="n"/>
+      <c r="E76" s="16" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="22" t="n"/>
+      <c r="B77" s="15" t="n"/>
+      <c r="C77" s="15" t="n"/>
+      <c r="D77" s="15" t="n"/>
+      <c r="E77" s="16" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="22" t="n"/>
+      <c r="B78" s="15" t="n"/>
+      <c r="C78" s="15" t="n"/>
+      <c r="D78" s="15" t="n"/>
+      <c r="E78" s="16" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="22" t="n"/>
+      <c r="B79" s="15" t="n"/>
+      <c r="C79" s="15" t="n"/>
+      <c r="D79" s="15" t="n"/>
+      <c r="E79" s="16" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B5:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=CATEGORIAS!$A$5:$A$15</formula1>
+    <dataValidation sqref="B6:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=CATEGORIAS!$A$6:$A$16</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D6:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Entrada,Saída"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>